<commit_message>
arreglado error de send email
</commit_message>
<xml_diff>
--- a/RPA-EOI/excel/Receta.xlsx
+++ b/RPA-EOI/excel/Receta.xlsx
@@ -28,49 +28,91 @@
     <x:t>nombre</x:t>
   </x:si>
   <x:si>
-    <x:t>4 comensales, 15m, Plato principal, Dificultad baja</x:t>
+    <x:t>8 comensales, 45m, Plato principal, Dificultad baja</x:t>
   </x:si>
   <x:si>
     <x:t>1</x:t>
   </x:si>
   <x:si>
-    <x:t>chorro de aceite de oliva</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Receta de Ensalada de gulas y gambas</x:t>
+    <x:t>Pollo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Receta de Arroz con pollo</x:t>
   </x:si>
   <x:si>
     <x:t/>
   </x:si>
   <x:si>
+    <x:t>kilogramo de Arroz blanco</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Cebolla</x:t>
+  </x:si>
+  <x:si>
+    <x:t>¼</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Ajoporro</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Pimentón rojo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Pimentón verde</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4</x:t>
+  </x:si>
+  <x:si>
+    <x:t>dientes de Ajo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Tomate</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Zanahoria</x:t>
+  </x:si>
+  <x:si>
+    <x:t>lata de Guisantes</x:t>
+  </x:si>
+  <x:si>
+    <x:t>lata de Maíz</x:t>
+  </x:si>
+  <x:si>
+    <x:t>½</x:t>
+  </x:si>
+  <x:si>
+    <x:t>taza de Aceite</x:t>
+  </x:si>
+  <x:si>
+    <x:t>cucharada sopera de Mostaza</x:t>
+  </x:si>
+  <x:si>
     <x:t>2</x:t>
   </x:si>
   <x:si>
-    <x:t>guindillas secas de cayena</x:t>
-  </x:si>
-  <x:si>
-    <x:t>300</x:t>
-  </x:si>
-  <x:si>
-    <x:t>gramos de gambas peladas</x:t>
-  </x:si>
-  <x:si>
-    <x:t>gramos de gulas</x:t>
-  </x:si>
-  <x:si>
-    <x:t>lata de mejillones al natural (de unos 120 g)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>100</x:t>
-  </x:si>
-  <x:si>
-    <x:t>gramos de canónigos</x:t>
-  </x:si>
-  <x:si>
-    <x:t>granada</x:t>
-  </x:si>
-  <x:si>
-    <x:t>pizca de sal</x:t>
+    <x:t>cucharadas soperas de Salsa inglesa</x:t>
+  </x:si>
+  <x:si>
+    <x:t>cucharadita de Orégano en polvo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>cucharadita de Comino</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10</x:t>
+  </x:si>
+  <x:si>
+    <x:t>tazas de Agua                                                                    (2400 mililitros)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Cubitos de caldo de pollo concentrado</x:t>
+  </x:si>
+  <x:si>
+    <x:t>cucharadita de Colorante alimentario</x:t>
+  </x:si>
+  <x:si>
+    <x:t>pizca de Sal y Pimienta</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -421,7 +463,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:D9"/>
+  <x:dimension ref="A1:D21"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:4">
@@ -457,10 +499,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
         <x:v>9</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>10</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
         <x:v>8</x:v>
@@ -471,10 +513,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
         <x:v>8</x:v>
@@ -488,7 +530,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
         <x:v>8</x:v>
@@ -502,7 +544,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
         <x:v>8</x:v>
@@ -513,10 +555,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
         <x:v>8</x:v>
@@ -527,10 +569,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>5</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
         <x:v>8</x:v>
@@ -544,9 +586,177 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:4">
+      <x:c r="A10" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="D9" s="0" t="s">
+      <x:c r="D10" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:4">
+      <x:c r="A11" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C11" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D11" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:4">
+      <x:c r="A12" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B12" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C12" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D12" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:4">
+      <x:c r="A13" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B13" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="C13" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="D13" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:4">
+      <x:c r="A14" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B14" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C14" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="D14" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" spans="1:4">
+      <x:c r="A15" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B15" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C15" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D15" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" spans="1:4">
+      <x:c r="A16" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B16" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="C16" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="D16" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" spans="1:4">
+      <x:c r="A17" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B17" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="C17" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="D17" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" spans="1:4">
+      <x:c r="A18" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B18" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="C18" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D18" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" spans="1:4">
+      <x:c r="A19" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B19" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C19" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="D19" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" spans="1:4">
+      <x:c r="A20" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B20" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C20" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="D20" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" spans="1:4">
+      <x:c r="A21" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B21" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C21" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="D21" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
     </x:row>

</xml_diff>